<commit_message>
Client update, Proposal Creation and Download
</commit_message>
<xml_diff>
--- a/AryamanBMS/wwwroot/templates/SalaryTemplate.xlsx
+++ b/AryamanBMS/wwwroot/templates/SalaryTemplate.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODING\ARYAMAN\AryamanBMS\AryamanBMS\AryamanBMS\wwwroot\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08570F7-22C7-4405-93E0-93F918465464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="20055" windowHeight="7440"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Salary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -165,12 +171,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,7 +324,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -343,18 +349,10 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -406,9 +404,6 @@
     <xf numFmtId="3" fontId="2" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -431,13 +426,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -475,7 +478,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -509,6 +512,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -543,9 +547,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -718,78 +723,78 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="9.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="25"/>
-    <col min="6" max="6" width="10.7109375" style="16" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" style="16"/>
-    <col min="9" max="9" width="11.42578125" style="16" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="16" customWidth="1"/>
-    <col min="11" max="11" width="10" style="16" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="16" customWidth="1"/>
-    <col min="13" max="13" width="9.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" style="16" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" style="16" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" style="16" customWidth="1"/>
-    <col min="17" max="17" width="17.85546875" style="16" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="16"/>
-    <col min="19" max="19" width="9.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.140625" style="16"/>
-    <col min="21" max="21" width="19.85546875" style="16" customWidth="1"/>
-    <col min="22" max="22" width="18.5703125" style="16" customWidth="1"/>
-    <col min="23" max="23" width="9.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.42578125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="21"/>
+    <col min="6" max="6" width="10.7265625" style="12" customWidth="1"/>
+    <col min="7" max="7" width="9.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" style="12"/>
+    <col min="9" max="9" width="11.453125" style="12" customWidth="1"/>
+    <col min="10" max="10" width="10.7265625" style="12" customWidth="1"/>
+    <col min="11" max="11" width="10" style="12" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" style="12" customWidth="1"/>
+    <col min="13" max="13" width="9.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.7265625" style="12" customWidth="1"/>
+    <col min="15" max="15" width="16.7265625" style="12" customWidth="1"/>
+    <col min="16" max="16" width="14.7265625" style="12" customWidth="1"/>
+    <col min="17" max="17" width="17.81640625" style="12" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="12"/>
+    <col min="19" max="19" width="9.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.1796875" style="12"/>
+    <col min="21" max="21" width="19.81640625" style="12" customWidth="1"/>
+    <col min="22" max="22" width="18.54296875" style="12" customWidth="1"/>
+    <col min="23" max="23" width="9.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.453125" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="18.75">
-      <c r="A1" s="42" t="s">
+    <row r="1" spans="1:27" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
-      <c r="V1" s="42"/>
-      <c r="W1" s="42"/>
-      <c r="X1" s="42"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="37"/>
+      <c r="X1" s="37"/>
       <c r="AA1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:27">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="O2" s="39"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="41"/>
-      <c r="T2" s="17"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="36"/>
+      <c r="T2" s="13"/>
       <c r="AA2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:27" s="15" customFormat="1" ht="45">
+    <row r="3" spans="1:27" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -799,64 +804,64 @@
       <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="K3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="Q3" s="19" t="s">
+      <c r="Q3" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="19" t="s">
+      <c r="R3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="S3" s="20" t="s">
+      <c r="S3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="T3" s="18" t="s">
+      <c r="T3" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="U3" s="19" t="s">
+      <c r="U3" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="V3" s="19" t="s">
+      <c r="V3" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="W3" s="19" t="s">
+      <c r="W3" s="15" t="s">
         <v>15</v>
       </c>
       <c r="X3" s="3" t="s">
@@ -866,7 +871,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -876,77 +881,77 @@
       <c r="C4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="17">
         <v>40550</v>
       </c>
-      <c r="E4" s="27">
+      <c r="E4" s="23">
         <v>26</v>
       </c>
-      <c r="F4" s="29">
+      <c r="F4" s="25">
         <f>D4/31*E4</f>
         <v>34009.677419354834</v>
       </c>
-      <c r="G4" s="30">
+      <c r="G4" s="26">
         <f>ROUND(F4*50%,0)</f>
         <v>17005</v>
       </c>
-      <c r="H4" s="30">
+      <c r="H4" s="26">
         <f>ROUND(G4*40%,0)</f>
         <v>6802</v>
       </c>
-      <c r="I4" s="30">
+      <c r="I4" s="26">
         <f>ROUND(G4*25%,0)</f>
         <v>4251</v>
       </c>
-      <c r="J4" s="30">
+      <c r="J4" s="26">
         <f>ROUND(G4*15%,0)</f>
         <v>2551</v>
       </c>
-      <c r="K4" s="30">
+      <c r="K4" s="26">
         <f>ROUND(G4*10%,0)</f>
         <v>1701</v>
       </c>
-      <c r="L4" s="31">
+      <c r="L4" s="27">
         <f>ROUND(G4*10%,0)</f>
         <v>1701</v>
       </c>
-      <c r="M4" s="32">
+      <c r="M4" s="28">
         <f>ROUND(SUM(G4:L4),0)</f>
         <v>34011</v>
       </c>
-      <c r="N4" s="32">
+      <c r="N4" s="28">
         <f>ROUND(M4-I4,0)</f>
         <v>29760</v>
       </c>
-      <c r="O4" s="33">
+      <c r="O4" s="29">
         <f>ROUND(IF(N4&lt;=15000,N4*12%,1800),0)</f>
         <v>1800</v>
       </c>
-      <c r="P4" s="34">
+      <c r="P4" s="30">
         <f>ROUNDUP(IF(G4&lt;=21000,G4*0.75%,0),0)</f>
         <v>128</v>
       </c>
-      <c r="Q4" s="35">
+      <c r="Q4" s="31">
         <f>IF(OR(AND(X4="Male",F4&gt;10000),AND(X4="Female",F4&gt;25000)),200,0)</f>
         <v>200</v>
       </c>
-      <c r="R4" s="30">
+      <c r="R4" s="26">
         <v>0</v>
       </c>
-      <c r="S4" s="36">
+      <c r="S4" s="32">
         <f>ROUND(M4-O4-P4-Q4-R4,0)</f>
         <v>31883</v>
       </c>
-      <c r="T4" s="29"/>
-      <c r="U4" s="33">
+      <c r="T4" s="25"/>
+      <c r="U4" s="29">
         <f>ROUND(IF(N4&lt;=15000,N4*13%,1950),0)</f>
         <v>1950</v>
       </c>
-      <c r="V4" s="34">
+      <c r="V4" s="30">
         <f>ROUNDUP(IF(G4&lt;=21000,G4*3.25%,0),0)</f>
         <v>553</v>
       </c>
-      <c r="W4" s="29">
+      <c r="W4" s="25">
         <f t="shared" ref="W4:W12" si="0">M4+U4+V4</f>
         <v>36514</v>
       </c>
@@ -954,7 +959,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -964,77 +969,77 @@
       <c r="C5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="18">
         <v>50050</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="23">
         <v>31</v>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="25">
         <f t="shared" ref="F5:F11" si="1">D5/31*E5</f>
         <v>50050</v>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="26">
         <f t="shared" ref="G5:G12" si="2">ROUND(F5*50%,0)</f>
         <v>25025</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="26">
         <f t="shared" ref="H5:H12" si="3">ROUND(G5*40%,0)</f>
         <v>10010</v>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="26">
         <f t="shared" ref="I5:I12" si="4">ROUND(G5*25%,0)</f>
         <v>6256</v>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="26">
         <f t="shared" ref="J5:J12" si="5">ROUND(G5*15%,0)</f>
         <v>3754</v>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="26">
         <f t="shared" ref="K5:K12" si="6">ROUND(G5*10%,0)</f>
         <v>2503</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="27">
         <f t="shared" ref="L5:L12" si="7">ROUND(G5*10%,0)</f>
         <v>2503</v>
       </c>
-      <c r="M5" s="32">
+      <c r="M5" s="28">
         <f t="shared" ref="M5:M12" si="8">ROUND(SUM(G5:L5),0)</f>
         <v>50051</v>
       </c>
-      <c r="N5" s="32">
+      <c r="N5" s="28">
         <f t="shared" ref="N5:N12" si="9">ROUND(M5-I5,0)</f>
         <v>43795</v>
       </c>
-      <c r="O5" s="33">
+      <c r="O5" s="29">
         <f t="shared" ref="O5:O12" si="10">ROUND(IF(N5&lt;=15000,N5*12%,1800),0)</f>
         <v>1800</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="30">
         <f t="shared" ref="P5:P12" si="11">ROUNDUP(IF(G5&lt;=21000,G5*0.75%,0),0)</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="35">
+      <c r="Q5" s="31">
         <f t="shared" ref="Q5:Q11" si="12">IF(OR(AND(X5="Male",F5&gt;10000),AND(X5="Female",F5&gt;25000)),200,0)</f>
         <v>200</v>
       </c>
-      <c r="R5" s="30">
+      <c r="R5" s="26">
         <v>0</v>
       </c>
-      <c r="S5" s="36">
+      <c r="S5" s="32">
         <f t="shared" ref="S5:S11" si="13">ROUND(M5-O5-P5-Q5-R5,0)</f>
         <v>48051</v>
       </c>
-      <c r="T5" s="29"/>
-      <c r="U5" s="33">
+      <c r="T5" s="25"/>
+      <c r="U5" s="29">
         <f t="shared" ref="U5:U12" si="14">ROUND(IF(N5&lt;=15000,N5*13%,1950),0)</f>
         <v>1950</v>
       </c>
-      <c r="V5" s="34">
+      <c r="V5" s="30">
         <f t="shared" ref="V5:V12" si="15">ROUNDUP(IF(G5&lt;=21000,G5*3.25%,0),0)</f>
         <v>0</v>
       </c>
-      <c r="W5" s="29">
+      <c r="W5" s="25">
         <f t="shared" si="0"/>
         <v>52001</v>
       </c>
@@ -1042,7 +1047,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:27">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -1052,77 +1057,77 @@
       <c r="C6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="17">
         <v>40550</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="23">
         <v>31</v>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="25">
         <f t="shared" si="1"/>
         <v>40550</v>
       </c>
-      <c r="G6" s="30">
+      <c r="G6" s="26">
         <f t="shared" si="2"/>
         <v>20275</v>
       </c>
-      <c r="H6" s="30">
+      <c r="H6" s="26">
         <f t="shared" si="3"/>
         <v>8110</v>
       </c>
-      <c r="I6" s="30">
+      <c r="I6" s="26">
         <f t="shared" si="4"/>
         <v>5069</v>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="26">
         <f t="shared" si="5"/>
         <v>3041</v>
       </c>
-      <c r="K6" s="30">
+      <c r="K6" s="26">
         <f t="shared" si="6"/>
         <v>2028</v>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="27">
         <f t="shared" si="7"/>
         <v>2028</v>
       </c>
-      <c r="M6" s="32">
+      <c r="M6" s="28">
         <f t="shared" si="8"/>
         <v>40551</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="28">
         <f t="shared" si="9"/>
         <v>35482</v>
       </c>
-      <c r="O6" s="33">
+      <c r="O6" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P6" s="34">
+      <c r="P6" s="30">
         <f t="shared" si="11"/>
         <v>153</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="31">
         <f t="shared" si="12"/>
         <v>200</v>
       </c>
-      <c r="R6" s="30">
+      <c r="R6" s="26">
         <v>0</v>
       </c>
-      <c r="S6" s="36">
+      <c r="S6" s="32">
         <f t="shared" si="13"/>
         <v>38398</v>
       </c>
-      <c r="T6" s="29"/>
-      <c r="U6" s="33">
+      <c r="T6" s="25"/>
+      <c r="U6" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V6" s="34">
+      <c r="V6" s="30">
         <f t="shared" si="15"/>
         <v>659</v>
       </c>
-      <c r="W6" s="29">
+      <c r="W6" s="25">
         <f t="shared" si="0"/>
         <v>43160</v>
       </c>
@@ -1130,7 +1135,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -1140,77 +1145,77 @@
       <c r="C7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="19">
         <v>28050</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="23">
         <v>31</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="25">
         <f t="shared" si="1"/>
         <v>28050</v>
       </c>
-      <c r="G7" s="30">
+      <c r="G7" s="26">
         <f t="shared" si="2"/>
         <v>14025</v>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="26">
         <f t="shared" si="3"/>
         <v>5610</v>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="26">
         <f t="shared" si="4"/>
         <v>3506</v>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="26">
         <f t="shared" si="5"/>
         <v>2104</v>
       </c>
-      <c r="K7" s="30">
+      <c r="K7" s="26">
         <f t="shared" si="6"/>
         <v>1403</v>
       </c>
-      <c r="L7" s="31">
+      <c r="L7" s="27">
         <f t="shared" si="7"/>
         <v>1403</v>
       </c>
-      <c r="M7" s="32">
+      <c r="M7" s="28">
         <f t="shared" si="8"/>
         <v>28051</v>
       </c>
-      <c r="N7" s="32">
+      <c r="N7" s="28">
         <f t="shared" si="9"/>
         <v>24545</v>
       </c>
-      <c r="O7" s="33">
+      <c r="O7" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P7" s="34">
+      <c r="P7" s="30">
         <f t="shared" si="11"/>
         <v>106</v>
       </c>
-      <c r="Q7" s="35">
+      <c r="Q7" s="31">
         <f t="shared" si="12"/>
         <v>200</v>
       </c>
-      <c r="R7" s="30">
+      <c r="R7" s="26">
         <v>0</v>
       </c>
-      <c r="S7" s="36">
+      <c r="S7" s="32">
         <f t="shared" si="13"/>
         <v>25945</v>
       </c>
-      <c r="T7" s="29"/>
-      <c r="U7" s="33">
+      <c r="T7" s="25"/>
+      <c r="U7" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V7" s="34">
+      <c r="V7" s="30">
         <f t="shared" si="15"/>
         <v>456</v>
       </c>
-      <c r="W7" s="29">
+      <c r="W7" s="25">
         <f t="shared" si="0"/>
         <v>30457</v>
       </c>
@@ -1218,351 +1223,351 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="19">
         <v>15000</v>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="23">
         <v>31</v>
       </c>
-      <c r="F8" s="29">
+      <c r="F8" s="25">
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
-      <c r="G8" s="30">
+      <c r="G8" s="26">
         <f t="shared" si="2"/>
         <v>7500</v>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="26">
         <f t="shared" si="3"/>
         <v>3000</v>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="26">
         <f t="shared" si="4"/>
         <v>1875</v>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="26">
         <f t="shared" si="5"/>
         <v>1125</v>
       </c>
-      <c r="K8" s="30">
+      <c r="K8" s="26">
         <f t="shared" si="6"/>
         <v>750</v>
       </c>
-      <c r="L8" s="31">
+      <c r="L8" s="27">
         <f t="shared" si="7"/>
         <v>750</v>
       </c>
-      <c r="M8" s="32">
+      <c r="M8" s="28">
         <f t="shared" si="8"/>
         <v>15000</v>
       </c>
-      <c r="N8" s="32">
+      <c r="N8" s="28">
         <f t="shared" si="9"/>
         <v>13125</v>
       </c>
-      <c r="O8" s="33">
+      <c r="O8" s="29">
         <f t="shared" si="10"/>
         <v>1575</v>
       </c>
-      <c r="P8" s="34">
+      <c r="P8" s="30">
         <f t="shared" si="11"/>
         <v>57</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="31">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="R8" s="30">
+      <c r="R8" s="26">
         <v>0</v>
       </c>
-      <c r="S8" s="36">
+      <c r="S8" s="32">
         <f t="shared" si="13"/>
         <v>13368</v>
       </c>
-      <c r="T8" s="37"/>
-      <c r="U8" s="33">
+      <c r="T8" s="25"/>
+      <c r="U8" s="29">
         <f t="shared" si="14"/>
         <v>1706</v>
       </c>
-      <c r="V8" s="34">
+      <c r="V8" s="30">
         <f t="shared" si="15"/>
         <v>244</v>
       </c>
-      <c r="W8" s="29">
+      <c r="W8" s="25">
         <f t="shared" si="0"/>
         <v>16950</v>
       </c>
-      <c r="X8" s="11" t="s">
+      <c r="X8" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="19">
         <v>32050</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="23">
         <v>31</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="25">
         <f t="shared" si="1"/>
         <v>32049.999999999996</v>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="26">
         <f t="shared" si="2"/>
         <v>16025</v>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="26">
         <f t="shared" si="3"/>
         <v>6410</v>
       </c>
-      <c r="I9" s="30">
+      <c r="I9" s="26">
         <f t="shared" si="4"/>
         <v>4006</v>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="26">
         <f t="shared" si="5"/>
         <v>2404</v>
       </c>
-      <c r="K9" s="30">
+      <c r="K9" s="26">
         <f t="shared" si="6"/>
         <v>1603</v>
       </c>
-      <c r="L9" s="31">
+      <c r="L9" s="27">
         <f t="shared" si="7"/>
         <v>1603</v>
       </c>
-      <c r="M9" s="32">
+      <c r="M9" s="28">
         <f t="shared" si="8"/>
         <v>32051</v>
       </c>
-      <c r="N9" s="32">
+      <c r="N9" s="28">
         <f t="shared" si="9"/>
         <v>28045</v>
       </c>
-      <c r="O9" s="33">
+      <c r="O9" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P9" s="34">
+      <c r="P9" s="30">
         <f t="shared" si="11"/>
         <v>121</v>
       </c>
-      <c r="Q9" s="35">
+      <c r="Q9" s="31">
         <f t="shared" si="12"/>
         <v>200</v>
       </c>
-      <c r="R9" s="30">
+      <c r="R9" s="26">
         <v>0</v>
       </c>
-      <c r="S9" s="36">
+      <c r="S9" s="32">
         <f t="shared" si="13"/>
         <v>29930</v>
       </c>
-      <c r="T9" s="37"/>
-      <c r="U9" s="33">
+      <c r="T9" s="25"/>
+      <c r="U9" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V9" s="34">
+      <c r="V9" s="30">
         <f t="shared" si="15"/>
         <v>521</v>
       </c>
-      <c r="W9" s="29">
+      <c r="W9" s="25">
         <f t="shared" si="0"/>
         <v>34522</v>
       </c>
-      <c r="X9" s="11" t="s">
+      <c r="X9" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:27">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="19">
         <v>22050</v>
       </c>
-      <c r="E10" s="27">
+      <c r="E10" s="23">
         <v>31</v>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="25">
         <f t="shared" si="1"/>
         <v>22050</v>
       </c>
-      <c r="G10" s="30">
+      <c r="G10" s="26">
         <f t="shared" si="2"/>
         <v>11025</v>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="26">
         <f t="shared" si="3"/>
         <v>4410</v>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="26">
         <f t="shared" si="4"/>
         <v>2756</v>
       </c>
-      <c r="J10" s="30">
+      <c r="J10" s="26">
         <f t="shared" si="5"/>
         <v>1654</v>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="26">
         <f t="shared" si="6"/>
         <v>1103</v>
       </c>
-      <c r="L10" s="31">
+      <c r="L10" s="27">
         <f t="shared" si="7"/>
         <v>1103</v>
       </c>
-      <c r="M10" s="32">
+      <c r="M10" s="28">
         <f t="shared" si="8"/>
         <v>22051</v>
       </c>
-      <c r="N10" s="32">
+      <c r="N10" s="28">
         <f t="shared" si="9"/>
         <v>19295</v>
       </c>
-      <c r="O10" s="33">
+      <c r="O10" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P10" s="34">
+      <c r="P10" s="30">
         <f t="shared" si="11"/>
         <v>83</v>
       </c>
-      <c r="Q10" s="35">
+      <c r="Q10" s="31">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="R10" s="30">
+      <c r="R10" s="26">
         <v>0</v>
       </c>
-      <c r="S10" s="36">
+      <c r="S10" s="32">
         <f t="shared" si="13"/>
         <v>20168</v>
       </c>
-      <c r="T10" s="37"/>
-      <c r="U10" s="33">
+      <c r="T10" s="25"/>
+      <c r="U10" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V10" s="34">
+      <c r="V10" s="30">
         <f t="shared" si="15"/>
         <v>359</v>
       </c>
-      <c r="W10" s="29">
+      <c r="W10" s="25">
         <f t="shared" si="0"/>
         <v>24360</v>
       </c>
-      <c r="X10" s="11" t="s">
+      <c r="X10" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:27">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="19">
         <v>40550</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="23">
         <v>31</v>
       </c>
-      <c r="F11" s="29">
+      <c r="F11" s="25">
         <f t="shared" si="1"/>
         <v>40550</v>
       </c>
-      <c r="G11" s="30">
+      <c r="G11" s="26">
         <f t="shared" si="2"/>
         <v>20275</v>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="26">
         <f t="shared" si="3"/>
         <v>8110</v>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="26">
         <f t="shared" si="4"/>
         <v>5069</v>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="26">
         <f t="shared" si="5"/>
         <v>3041</v>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="26">
         <f t="shared" si="6"/>
         <v>2028</v>
       </c>
-      <c r="L11" s="31">
+      <c r="L11" s="27">
         <f t="shared" si="7"/>
         <v>2028</v>
       </c>
-      <c r="M11" s="32">
+      <c r="M11" s="28">
         <f t="shared" si="8"/>
         <v>40551</v>
       </c>
-      <c r="N11" s="32">
+      <c r="N11" s="28">
         <f t="shared" si="9"/>
         <v>35482</v>
       </c>
-      <c r="O11" s="33">
+      <c r="O11" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="30">
         <f t="shared" si="11"/>
         <v>153</v>
       </c>
-      <c r="Q11" s="35">
+      <c r="Q11" s="31">
         <f t="shared" si="12"/>
         <v>200</v>
       </c>
-      <c r="R11" s="30">
+      <c r="R11" s="26">
         <v>0</v>
       </c>
-      <c r="S11" s="36">
+      <c r="S11" s="32">
         <f t="shared" si="13"/>
         <v>38398</v>
       </c>
-      <c r="T11" s="29"/>
-      <c r="U11" s="33">
+      <c r="T11" s="25"/>
+      <c r="U11" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V11" s="34">
+      <c r="V11" s="30">
         <f t="shared" si="15"/>
         <v>659</v>
       </c>
-      <c r="W11" s="29">
+      <c r="W11" s="25">
         <f t="shared" si="0"/>
         <v>43160</v>
       </c>
@@ -1570,77 +1575,77 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:27">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="20">
         <f t="shared" ref="D12:E12" si="16">SUM(D4:D11)</f>
         <v>268850</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="24">
         <f t="shared" si="16"/>
         <v>243</v>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="25">
         <f>SUM(F4:F11)</f>
         <v>262309.67741935485</v>
       </c>
-      <c r="G12" s="30">
+      <c r="G12" s="26">
         <f t="shared" si="2"/>
         <v>131155</v>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="26">
         <f t="shared" si="3"/>
         <v>52462</v>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="26">
         <f t="shared" si="4"/>
         <v>32789</v>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="26">
         <f t="shared" si="5"/>
         <v>19673</v>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="26">
         <f t="shared" si="6"/>
         <v>13116</v>
       </c>
-      <c r="L12" s="31">
+      <c r="L12" s="27">
         <f t="shared" si="7"/>
         <v>13116</v>
       </c>
-      <c r="M12" s="32">
+      <c r="M12" s="28">
         <f t="shared" si="8"/>
         <v>262311</v>
       </c>
-      <c r="N12" s="32">
+      <c r="N12" s="28">
         <f t="shared" si="9"/>
         <v>229522</v>
       </c>
-      <c r="O12" s="33">
+      <c r="O12" s="29">
         <f t="shared" si="10"/>
         <v>1800</v>
       </c>
-      <c r="P12" s="34">
+      <c r="P12" s="30">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="35"/>
-      <c r="R12" s="30"/>
-      <c r="S12" s="36"/>
-      <c r="T12" s="38"/>
-      <c r="U12" s="33">
+      <c r="Q12" s="31"/>
+      <c r="R12" s="26"/>
+      <c r="S12" s="32"/>
+      <c r="T12" s="33"/>
+      <c r="U12" s="29">
         <f t="shared" si="14"/>
         <v>1950</v>
       </c>
-      <c r="V12" s="34">
+      <c r="V12" s="30">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="W12" s="29">
+      <c r="W12" s="25">
         <f t="shared" si="0"/>
         <v>264261</v>
       </c>
@@ -1652,7 +1657,7 @@
     <mergeCell ref="A1:X1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong Format" error="Max  Length 40  Letters&#10;&#10;Please do not use dots ( . )  in Beneficary Name like &quot;PVT. LTD.&quot;" promptTitle="Baneficiry Account Name" prompt="Max  Length 40  Letters&#10;&#10;Please do not use dots ( . )  in Beneficary Name like &quot;PVT. LTD.&quot;" sqref="C4:C5 C8:C11">
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong Format" error="Max  Length 40  Letters_x000a__x000a_Please do not use dots ( . )  in Beneficary Name like &quot;PVT. LTD.&quot;" promptTitle="Baneficiry Account Name" prompt="Max  Length 40  Letters_x000a__x000a_Please do not use dots ( . )  in Beneficary Name like &quot;PVT. LTD.&quot;" sqref="C4:C5 C8:C11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>40</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>